<commit_message>
Add source-local specimen header inheritance
</commit_message>
<xml_diff>
--- a/tests/fixtures/source/FX-004-warning-cells.xlsx
+++ b/tests/fixtures/source/FX-004-warning-cells.xlsx
@@ -403,13 +403,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v/>
+        <v>Synthetic Sample A</v>
       </c>
       <c r="B1" t="str">
         <v>Merged Synthetic Sample</v>
       </c>
       <c r="C1" t="str">
-        <v>Synthetic Sample C</v>
+        <v/>
       </c>
     </row>
     <row r="2">

</xml_diff>